<commit_message>
Update of example input files and terms in translation tables, optimization of scripts for standardizing taxon and location names, change of column name verbatimTaxonRank to originalNameUsage
</commit_message>
<xml_diff>
--- a/Config/DatabaseInfo.xlsx
+++ b/Config/DatabaseInfo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhD\1. Data paper\SInAS_github\SInAS\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7594C5-4626-4683-8EE1-01CDA2D20602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83A5033-98BD-408A-AF46-56EED49C5D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="95">
   <si>
     <t>Dataset_brief_name</t>
   </si>
@@ -250,18 +250,9 @@
     <t>GAVIA_taxon_region_list_example.xlsx</t>
   </si>
   <si>
-    <t>GRIIS_sTwist_Hanno_Aug92019_resend_example.xlsx</t>
-  </si>
-  <si>
     <t>GloNAF_taxon_region_list_example.xlsx</t>
   </si>
   <si>
-    <t>GlobalAlienSpeciesFirstRecordDatabase_v1.2_withcountries_example.xlsx</t>
-  </si>
-  <si>
-    <t>Author</t>
-  </si>
-  <si>
     <t>Dataset_scope</t>
   </si>
   <si>
@@ -311,6 +302,24 @@
   </si>
   <si>
     <t>IUCN. The IUCN Red List of Threatened Species. https://www.iucnredlist.org (v. 2024-2)</t>
+  </si>
+  <si>
+    <t>GlobalAlienSpeciesFirstRecordDatabase_v3.1_freedata_example.xlsx</t>
+  </si>
+  <si>
+    <t>GRIIS - Country Compendium V1_0_example.csv</t>
+  </si>
+  <si>
+    <t>occurrenceStatus</t>
+  </si>
+  <si>
+    <t>isInvasive</t>
+  </si>
+  <si>
+    <t>TaxonName</t>
+  </si>
+  <si>
+    <t>Pathway</t>
   </si>
 </sst>
 </file>
@@ -686,7 +695,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -745,20 +754,18 @@
         <v>35</v>
       </c>
       <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
         <v>73</v>
-      </c>
-      <c r="C2" t="s">
-        <v>76</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>74</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="G2" s="3"/>
       <c r="J2" t="s">
         <v>32</v>
       </c>
@@ -766,13 +773,16 @@
         <v>36</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="P2" t="s">
         <v>38</v>
       </c>
       <c r="Q2" t="s">
         <v>38</v>
+      </c>
+      <c r="R2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
@@ -780,10 +790,10 @@
         <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
         <v>25</v>
@@ -797,14 +807,17 @@
       <c r="J3" t="s">
         <v>26</v>
       </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
       <c r="N3" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
+      </c>
+      <c r="O3" t="s">
+        <v>91</v>
       </c>
       <c r="P3" t="s">
         <v>22</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>92</v>
       </c>
       <c r="S3" t="s">
         <v>27</v>
@@ -818,7 +831,7 @@
         <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
@@ -830,7 +843,7 @@
         <v>32</v>
       </c>
       <c r="N4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -838,10 +851,10 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
         <v>42</v>
@@ -856,7 +869,7 @@
         <v>45</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P5" t="s">
         <v>46</v>
@@ -870,7 +883,7 @@
         <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
         <v>49</v>
@@ -888,7 +901,7 @@
         <v>51</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="O6" t="s">
         <v>53</v>
@@ -905,37 +918,37 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
         <v>78</v>
-      </c>
-      <c r="B7" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E7" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" t="s">
-        <v>81</v>
       </c>
       <c r="I7" t="s">
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="P7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="S7" t="s">
         <v>27</v>

</xml_diff>